<commit_message>
Solved the problem for the billings sendto to the accounts team
</commit_message>
<xml_diff>
--- a/src/assets/importVendor.xlsx
+++ b/src/assets/importVendor.xlsx
@@ -1,14 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A99FD3F-D15E-42F9-B884-8DFE61E12B08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432"/>
   </bookViews>
   <sheets>
-    <sheet name="Vendor Master" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Vendor Master" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -50,35 +49,35 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FF000000"/>
+      <family val="2"/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FFCE9178"/>
-      <name val="Menlo"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="FFCE9178"/>
+      <family val="2"/>
+      <sz val="12"/>
+      <name val="Menlo"/>
     </font>
   </fonts>
   <fills count="3">
@@ -103,18 +102,10 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -466,9 +457,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J16"/>
-  <sheetFormatPr defaultColWidth="8.83984375" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.83984375" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="54.83984375" customWidth="1"/>
     <col min="2" max="2" width="53" customWidth="1"/>
@@ -480,7 +471,7 @@
     <col min="8" max="8" width="41" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -512,27 +503,27 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-    </row>
-    <row r="12" spans="1:10" ht="15.3">
-      <c r="A12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" ht="15.3">
-      <c r="A13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" ht="15.3">
-      <c r="A14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" ht="15.3">
-      <c r="A15" s="2"/>
-    </row>
-    <row r="16" spans="1:10" ht="15.3">
-      <c r="A16" s="2"/>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+    </row>
+    <row r="12" ht="15.3" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3"/>
+    </row>
+    <row r="13" ht="15.3" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3"/>
+    </row>
+    <row r="14" ht="15.3" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3"/>
+    </row>
+    <row r="15" ht="15.3" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="3"/>
+    </row>
+    <row r="16" ht="15.3" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>